<commit_message>
feat: daily expense ledger, soft-delete voided audit trail, and chartjs sales trends
</commit_message>
<xml_diff>
--- a/database_templates/Client_Template_Orders_and_Menu.xlsx
+++ b/database_templates/Client_Template_Orders_and_Menu.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Menu" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Orders" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Expenses" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -692,4 +693,127 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="23" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="31" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Expense_ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Timestamp</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>EXP-20261020-001</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 09:30:00</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Inventory</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Fresh Vegetables &amp; Herbs</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>1250</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>EXP-20261020-002</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 11:00:00</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Staff</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Kitchen Helper Daily Wages</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>EXP-20261020-003</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 16:15:00</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Commercial LPG Gas Cylinder</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>1850</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>